<commit_message>
Release v1.1.0: current-unit correction, revised figures, ablation results
- TIA-mode current columns rescaled by 1 MOhm / 27 kOhm (the logger assumed
  1 MOhm; the board TIA uses 27 kOhm); integrator-mode current columns renamed
  *_nominal because their integration capacitance is unverified
  (scripts/correct_currents_v110.py, worksheet-level edit).
- Fig. 4f: plot_fig4f.py and simulation_results/fig4f/fig4f_points.csv
  (Supplementary Table 2), pixel-identical to the submitted panel.
- Fig. 5d: plot_fig5d_operands.py replaces plot_fig5d_traffic.py (no ratio
  arrows; "Re-read baseline", "U-AIMDC"). Fig. 5e: plot_fig5e_memory.py.
- simulation_results/ablation_q1000/: Supplementary Note 6.4 / Table 14.
- README, CITATION, CHANGELOG: revised title and terminology, measurement
  interface and current units, session labels, figure index.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S5pjbGy8jaCckQTGg1VLSs
</commit_message>
<xml_diff>
--- a/4t2c_auto_dataset_0903.xlsx
+++ b/4t2c_auto_dataset_0903.xlsx
@@ -517,7 +517,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>MBL −1.5 V, BL 0 V, SL 차동, TIA CH8 (Rf 1 MΩ), 점당 3샘플</t>
+          <t>MBL −1.5 V, BL 0 V, SL 차동, TIA CH8 (Rf 27 kΩ; listed as 1 MΩ before v1.1.0), 점당 3샘플</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr"/>
@@ -569,7 +569,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>점당 표준오차 2.33 code (1 code = 1.221 mV = 1.221 nA)</t>
+          <t>점당 표준오차 2.33 code (1 code = 1.221 mV = 45.2 nA; 1.221 nA before v1.1.0, which assumed Rf = 1 MΩ)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr"/>
@@ -26616,7 +26616,7 @@
         <v>341.33</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.416768</v>
+        <v>15.4358519</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -26635,7 +26635,7 @@
         <v>370.67</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.452584</v>
+        <v>16.7623704</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -26654,7 +26654,7 @@
         <v>320.67</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.391534</v>
+        <v>14.5012593</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -26673,7 +26673,7 @@
         <v>392.67</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.479446</v>
+        <v>17.7572593</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
@@ -26692,7 +26692,7 @@
         <v>315.33</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.385022</v>
+        <v>14.2600741</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -26711,7 +26711,7 @@
         <v>425.33</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.519333</v>
+        <v>19.2345556</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
@@ -26730,7 +26730,7 @@
         <v>300.67</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.367114</v>
+        <v>13.5968148</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
@@ -26749,7 +26749,7 @@
         <v>451.67</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.551486</v>
+        <v>20.4254074</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
@@ -26768,7 +26768,7 @@
         <v>291.67</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.356125</v>
+        <v>13.1898148</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
@@ -26787,7 +26787,7 @@
         <v>488</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.595849</v>
+        <v>22.0684815</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
@@ -26806,7 +26806,7 @@
         <v>281.67</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.343915</v>
+        <v>12.7375926</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
@@ -26825,7 +26825,7 @@
         <v>519</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.6337</v>
+        <v>23.4703704</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
@@ -26844,7 +26844,7 @@
         <v>284.33</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.347171</v>
+        <v>12.8581852</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
@@ -26863,7 +26863,7 @@
         <v>291</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.355311</v>
+        <v>13.1596667</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
@@ -26882,7 +26882,7 @@
         <v>296.67</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.36223</v>
+        <v>13.4159259</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
@@ -26901,7 +26901,7 @@
         <v>310.67</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.379324</v>
+        <v>14.049037</v>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
@@ -26920,7 +26920,7 @@
         <v>328</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0.400488</v>
+        <v>14.8328889</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
@@ -26939,7 +26939,7 @@
         <v>348.33</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0.425315</v>
+        <v>15.7524074</v>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
@@ -26958,7 +26958,7 @@
         <v>369</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>0.450549</v>
+        <v>16.687</v>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
@@ -26977,7 +26977,7 @@
         <v>389.67</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0.475783</v>
+        <v>17.6215926</v>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
@@ -26996,7 +26996,7 @@
         <v>419</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0.5116000000000001</v>
+        <v>18.9481481</v>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
@@ -27015,7 +27015,7 @@
         <v>322.33</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0.393569</v>
+        <v>14.5766296</v>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
@@ -27034,7 +27034,7 @@
         <v>345.33</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0.421652</v>
+        <v>15.6167407</v>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
@@ -27053,7 +27053,7 @@
         <v>304.33</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.371591</v>
+        <v>13.7626296</v>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
@@ -27072,7 +27072,7 @@
         <v>373</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>0.455433</v>
+        <v>16.8678889</v>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
@@ -27091,7 +27091,7 @@
         <v>281.67</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0.343915</v>
+        <v>12.7375926</v>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
@@ -27110,7 +27110,7 @@
         <v>401</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.489621</v>
+        <v>18.1341111</v>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
@@ -27129,7 +27129,7 @@
         <v>276.67</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0.33781</v>
+        <v>12.5114815</v>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
@@ -27148,7 +27148,7 @@
         <v>429.33</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>0.524217</v>
+        <v>19.4154444</v>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
@@ -27167,7 +27167,7 @@
         <v>267.67</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0.326821</v>
+        <v>12.1044815</v>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
@@ -27186,7 +27186,7 @@
         <v>466</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>0.568987</v>
+        <v>21.0735926</v>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
@@ -27205,7 +27205,7 @@
         <v>260.67</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0.318274</v>
+        <v>11.7879259</v>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
@@ -27224,7 +27224,7 @@
         <v>493.33</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0.602361</v>
+        <v>22.3096667</v>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
@@ -27243,7 +27243,7 @@
         <v>260.33</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>0.317867</v>
+        <v>11.7728519</v>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
@@ -27262,7 +27262,7 @@
         <v>266</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>0.324786</v>
+        <v>12.0291111</v>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
@@ -27281,7 +27281,7 @@
         <v>272.33</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0.332519</v>
+        <v>12.3155185</v>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
@@ -27300,7 +27300,7 @@
         <v>285</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0.347985</v>
+        <v>12.8883333</v>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
@@ -27319,7 +27319,7 @@
         <v>305.67</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>0.373219</v>
+        <v>13.8229259</v>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
@@ -27338,7 +27338,7 @@
         <v>324.67</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>0.396418</v>
+        <v>14.6821481</v>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
@@ -27357,7 +27357,7 @@
         <v>351.67</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>0.429385</v>
+        <v>15.9031481</v>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
@@ -27376,7 +27376,7 @@
         <v>369.67</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>0.451363</v>
+        <v>16.7171481</v>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
@@ -27395,7 +27395,7 @@
         <v>399</v>
       </c>
       <c r="D43" s="2" t="n">
-        <v>0.487179</v>
+        <v>18.0436667</v>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>

</xml_diff>